<commit_message>
Corrida | SFE-PTOT | 2026-06-17 12:08:00.041477
</commit_message>
<xml_diff>
--- a/indicadores/SFE-PTOT_out.xlsx
+++ b/indicadores/SFE-PTOT_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2052,9 +2058,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2065,7 +2075,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2079,12 +2089,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.343167902977312</v>
+        <v>0.341882879900403</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2095,7 +2105,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2123,7 +2133,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2137,12 +2147,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.117764209633846</v>
+        <v>0.116883903568993</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2165,7 +2175,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2179,7 +2189,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2193,7 +2203,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2207,12 +2217,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.333551528207177</v>
+        <v>0.354380518732631</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2223,7 +2233,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2237,12 +2247,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0192025968068423</v>
+        <v>0.0175347994332439</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2385,10 +2395,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2401,10 +2411,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2428,66 +2438,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>573.063</v>
@@ -2540,7 +2550,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>568.072</v>
@@ -2597,7 +2607,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>619.209</v>
@@ -2654,7 +2664,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>644.954</v>
@@ -2711,7 +2721,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>665.599</v>
@@ -2768,7 +2778,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>609.383</v>
@@ -2825,7 +2835,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>653.401</v>
@@ -2882,7 +2892,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>661.063</v>
@@ -2939,7 +2949,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>582.993</v>
@@ -2996,7 +3006,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>622.185</v>
@@ -3053,7 +3063,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>657.793</v>
@@ -3110,7 +3120,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>837.965</v>
@@ -3167,7 +3177,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>703.382</v>
@@ -3226,7 +3236,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>643.721</v>
@@ -3285,7 +3295,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>779.418</v>
@@ -3344,7 +3354,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>719.814</v>
@@ -3403,7 +3413,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>748.166</v>
@@ -3462,7 +3472,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>771.173</v>
@@ -3521,7 +3531,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>851.873</v>
@@ -3580,7 +3590,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>818.92</v>
@@ -3639,7 +3649,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>806.648</v>
@@ -3698,7 +3708,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>841.847</v>
@@ -3757,7 +3767,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>819.444</v>
@@ -3816,7 +3826,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>894.444</v>
@@ -3875,7 +3885,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>810.039</v>
@@ -3934,7 +3944,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>796.084</v>
@@ -3993,7 +4003,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>926.243</v>
@@ -4052,7 +4062,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>962.366</v>
@@ -4111,7 +4121,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>968.002</v>
@@ -4170,7 +4180,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>888.268</v>
@@ -4229,7 +4239,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>933.905</v>
@@ -4288,7 +4298,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>926.313</v>
@@ -4347,7 +4357,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>881.051</v>
@@ -4406,7 +4416,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>928.681</v>
@@ -4465,7 +4475,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>875.295</v>
@@ -4524,7 +4534,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>950.837</v>
@@ -4583,7 +4593,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>887.05</v>
@@ -4642,7 +4652,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>851.599</v>
@@ -4701,7 +4711,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>965.025</v>
@@ -4760,7 +4770,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>954.488</v>
@@ -4819,7 +4829,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>1040.75</v>
@@ -4878,7 +4888,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>887.835</v>
@@ -4937,7 +4947,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>917.78</v>
@@ -4996,7 +5006,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>913.481</v>
@@ -5055,7 +5065,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>878.663</v>
@@ -5114,7 +5124,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>927.605</v>
@@ -5173,7 +5183,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>937.047</v>
@@ -5232,7 +5242,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>1010.118</v>
@@ -5291,7 +5301,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>947.314</v>
@@ -5350,7 +5360,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>860.744</v>
@@ -5409,7 +5419,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>1006.285</v>
@@ -5468,7 +5478,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>986.365</v>
@@ -5527,7 +5537,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>978.223</v>
@@ -5586,7 +5596,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>929.849</v>
@@ -5645,7 +5655,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>935.601</v>
@@ -5704,7 +5714,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>931.783</v>
@@ -5763,7 +5773,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>884.975</v>
@@ -5822,7 +5832,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>899.815</v>
@@ -5881,7 +5891,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>910.183</v>
@@ -5940,7 +5950,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>1042.295</v>
@@ -5999,7 +6009,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>971.628</v>
@@ -6058,7 +6068,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>865.954</v>
@@ -6117,7 +6127,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>979.217</v>
@@ -6176,7 +6186,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>1049.041</v>
@@ -6235,7 +6245,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>1075.28</v>
@@ -6294,7 +6304,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>945.764</v>
@@ -6353,7 +6363,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>982.254</v>
@@ -6412,7 +6422,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>977.903</v>
@@ -6471,7 +6481,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>894.485</v>
@@ -6530,7 +6540,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>893.295</v>
@@ -6589,7 +6599,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>919.585</v>
@@ -6648,7 +6658,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>933.153</v>
@@ -6707,7 +6717,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>843.662</v>
@@ -6766,7 +6776,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>798.858</v>
@@ -6825,7 +6835,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>946.645</v>
@@ -6884,7 +6894,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>888.615</v>
@@ -6943,7 +6953,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>934.603</v>
@@ -7002,7 +7012,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>854.1</v>
@@ -7061,7 +7071,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>904.683</v>
@@ -7120,7 +7130,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>870.836</v>
@@ -7179,7 +7189,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>847.459</v>
@@ -7238,7 +7248,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>876.11</v>
@@ -7297,7 +7307,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>868.83</v>
@@ -7356,7 +7366,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>924.139</v>
@@ -7415,7 +7425,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>916.241</v>
@@ -7474,7 +7484,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>861.275</v>
@@ -7533,7 +7543,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>1028.746</v>
@@ -7592,7 +7602,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>978.146</v>
@@ -7651,7 +7661,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>801.945</v>
@@ -7710,7 +7720,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>928.851</v>
@@ -7769,7 +7779,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>954.428</v>
@@ -7828,7 +7838,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>934.155</v>
@@ -7887,7 +7897,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>903.037</v>
@@ -7946,7 +7956,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>955.197</v>
@@ -8005,7 +8015,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>915.509</v>
@@ -8064,7 +8074,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>1003.37</v>
@@ -8123,7 +8133,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>1018.663</v>
@@ -8182,7 +8192,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>940.217</v>
@@ -8241,7 +8251,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>1098.733</v>
@@ -8300,7 +8310,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>1042.481</v>
@@ -8359,7 +8369,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>1077.417</v>
@@ -8418,7 +8428,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>1016.847</v>
@@ -8477,7 +8487,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>1050.808</v>
@@ -8536,7 +8546,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>1022.359</v>
@@ -8595,7 +8605,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>1010.092</v>
@@ -8654,7 +8664,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>1029.598</v>
@@ -8713,7 +8723,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>1026.693</v>
@@ -8772,7 +8782,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>1136.067</v>
@@ -8831,7 +8841,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>1065.79</v>
@@ -8890,7 +8900,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>999.797</v>
@@ -8949,7 +8959,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>1250.49</v>
@@ -9008,7 +9018,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>1178.212</v>
@@ -9067,7 +9077,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>1199.991</v>
@@ -9126,7 +9136,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>1084.113</v>
@@ -9185,7 +9195,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>1175.344</v>
@@ -9244,7 +9254,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>1153.475</v>
@@ -9303,7 +9313,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>1146.243</v>
@@ -9362,7 +9372,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>1168.693</v>
@@ -9421,7 +9431,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>1157.873</v>
@@ -9480,7 +9490,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>1241.211</v>
@@ -9539,7 +9549,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>1203.137</v>
@@ -9598,7 +9608,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>1071.033</v>
@@ -9657,7 +9667,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>1250.395</v>
@@ -9716,7 +9726,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>1267.466</v>
@@ -9775,7 +9785,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>1321.396</v>
@@ -9834,7 +9844,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>1135.338</v>
@@ -9893,7 +9903,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>1255.274</v>
@@ -9952,7 +9962,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>1268.004</v>
@@ -10011,7 +10021,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>1240.587</v>
@@ -10070,7 +10080,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>1270.548</v>
@@ -10129,7 +10139,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>1251.645</v>
@@ -10188,7 +10198,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>1264.636</v>
@@ -10247,7 +10257,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>1215.725</v>
@@ -10306,7 +10316,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>1137.238</v>
@@ -10365,7 +10375,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>1178.177</v>
@@ -10424,7 +10434,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>986.162</v>
@@ -10483,7 +10493,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>1404.672</v>
@@ -10542,7 +10552,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>1290.54</v>
@@ -10601,7 +10611,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>1380.748</v>
@@ -10660,7 +10670,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>1396.747</v>
@@ -10719,7 +10729,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>1348.153</v>
@@ -10778,7 +10788,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>1445.069</v>
@@ -10837,7 +10847,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>1444.547</v>
@@ -10896,7 +10906,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>1453.246</v>
@@ -10955,7 +10965,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>1440.599</v>
@@ -11014,7 +11024,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>1388.356</v>
@@ -11073,7 +11083,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>1362.847</v>
@@ -11132,7 +11142,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>1476.094</v>
@@ -11191,7 +11201,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>1358.507</v>
@@ -11250,7 +11260,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>1044.877</v>
@@ -11309,7 +11319,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>1518.785</v>
@@ -11368,7 +11378,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>1510.635</v>
@@ -11427,7 +11437,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>1432.119</v>
@@ -11486,7 +11496,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>1434.984</v>
@@ -11545,7 +11555,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>1335.359</v>
@@ -11604,7 +11614,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>1420.154</v>
@@ -11663,7 +11673,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>1363.264</v>
@@ -11722,7 +11732,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>1296.967</v>
@@ -11781,7 +11791,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>1435.192</v>
@@ -11840,7 +11850,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>1414.284</v>
@@ -11899,7 +11909,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>1396.553</v>
@@ -11958,7 +11968,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>1288.427</v>
@@ -12017,7 +12027,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>1281.97</v>
@@ -12076,7 +12086,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>1366.131</v>
@@ -12135,7 +12145,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>1319.895</v>
@@ -12194,7 +12204,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>1429.414</v>
@@ -12253,7 +12263,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>1329.016</v>
@@ -12312,7 +12322,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>1406.58</v>
@@ -12371,7 +12381,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>1370.593</v>
@@ -12430,7 +12440,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>1186.944</v>
@@ -12489,7 +12499,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>1360.137</v>
@@ -12548,7 +12558,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>1408.989</v>
@@ -12607,7 +12617,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>1442.807</v>
@@ -12666,7 +12676,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>1291.06487544394</v>
@@ -12725,7 +12735,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>1415.80605124822</v>
@@ -12784,7 +12794,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>1420.77561654041</v>
@@ -12843,7 +12853,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>1368.32216436675</v>
@@ -12902,7 +12912,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>1423.43659870296</v>
@@ -12961,7 +12971,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>1386.47548419421</v>
@@ -13020,7 +13030,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>1476.52337780863</v>
@@ -13079,7 +13089,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>1408.324</v>
@@ -13138,7 +13148,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>1408.324</v>
@@ -13197,7 +13207,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>1302.516</v>
@@ -13256,7 +13266,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>1458.387</v>
@@ -13315,7 +13325,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>1473.522</v>
@@ -13374,7 +13384,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>1460.466</v>
@@ -13433,7 +13443,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>1395.241</v>
@@ -13492,7 +13502,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>1544.037</v>
@@ -13551,7 +13561,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>1527.666</v>
@@ -13610,7 +13620,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>1525.406</v>
@@ -13669,7 +13679,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>1543.759</v>
@@ -13728,7 +13738,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>1522.193</v>
@@ -13787,7 +13797,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>1609.385</v>
@@ -13846,7 +13856,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>1450.329</v>
@@ -13905,7 +13915,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>1570.14</v>
@@ -13964,7 +13974,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>1566.443</v>
@@ -14023,7 +14033,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>1571.274</v>
@@ -14082,7 +14092,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>1494.221</v>
@@ -14141,7 +14151,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>1673.883</v>
@@ -14200,7 +14210,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>1555.659</v>
@@ -14259,7 +14269,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>1517.151</v>
@@ -14318,7 +14328,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>1584.43</v>
@@ -14377,7 +14387,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>1684.479</v>
@@ -14436,7 +14446,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>1590.722</v>
@@ -14495,7 +14505,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>1603.592</v>
@@ -14554,7 +14564,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>1463.343</v>
@@ -14613,7 +14623,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>1713.085</v>
@@ -14672,7 +14682,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>1644.378</v>
@@ -14731,7 +14741,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>1597.299</v>
@@ -14790,7 +14800,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>1523.941</v>
@@ -14849,7 +14859,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>1628.288</v>
@@ -14908,7 +14918,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>1556.546</v>
@@ -14967,7 +14977,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>1521.06</v>
@@ -15026,7 +15036,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>1621.724</v>
@@ -15085,7 +15095,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>1314.652</v>
@@ -15144,7 +15154,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>1450.4255</v>
@@ -15203,7 +15213,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>1586.199</v>
@@ -15262,7 +15272,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>1384.886</v>
@@ -15321,7 +15331,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>1588.157</v>
@@ -15380,7 +15390,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>1604.617</v>
@@ -15439,7 +15449,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>1652.613</v>
@@ -15498,7 +15508,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>1581.502</v>
@@ -15557,7 +15567,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>1596.766</v>
@@ -15616,7 +15626,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>1697.803</v>
@@ -15675,7 +15685,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>1385.775</v>
@@ -15734,7 +15744,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>1467.733</v>
@@ -15793,7 +15803,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>1375.799</v>
@@ -15852,7 +15862,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>1300.746</v>
@@ -15911,7 +15921,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>1272.297</v>
@@ -15970,7 +15980,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>1520.792</v>
@@ -16029,7 +16039,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>1596.548</v>
@@ -16088,7 +16098,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>1647.557</v>
@@ -16147,7 +16157,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>1581.575</v>
@@ -16206,7 +16216,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>1531.968</v>
@@ -16265,7 +16275,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>1668.293</v>
@@ -16324,7 +16334,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>1532.637</v>
@@ -16383,7 +16393,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>1534.626</v>
@@ -16442,7 +16452,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>1666.878</v>
@@ -16501,7 +16511,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>1602.64</v>
@@ -16560,7 +16570,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>1772.111</v>
@@ -16619,7 +16629,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>1787.028</v>
@@ -16678,7 +16688,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>1697.181</v>
@@ -16737,7 +16747,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>1807.224</v>
@@ -16796,7 +16806,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>1530.769</v>
@@ -16855,7 +16865,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>1735.332</v>
@@ -16914,7 +16924,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>1736.533</v>
@@ -16973,7 +16983,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>1853.94</v>
@@ -17032,7 +17042,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>1943.871</v>
@@ -17091,7 +17101,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>1731.316</v>
@@ -17150,7 +17160,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>1849.25</v>
@@ -17209,7 +17219,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>1872.561</v>
@@ -17268,7 +17278,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>1945.287</v>
@@ -17327,7 +17337,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>2018.013</v>
@@ -17386,7 +17396,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>1823.374</v>
@@ -17445,7 +17455,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>1961.579</v>
@@ -17504,7 +17514,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>1721.412</v>
@@ -17563,7 +17573,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>1743.143</v>
@@ -17622,7 +17632,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>1754.232</v>
@@ -17681,7 +17691,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>1836.504</v>
@@ -17740,7 +17750,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>1907.897</v>
@@ -17799,7 +17809,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>2007.526</v>
@@ -17858,7 +17868,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>1972.775</v>
@@ -17917,7 +17927,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>2045.782</v>
@@ -17976,7 +17986,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>1976.24</v>
@@ -18035,7 +18045,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>1909.739</v>
@@ -18094,7 +18104,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>1735.47</v>
@@ -18153,7 +18163,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>1766.002</v>
@@ -18212,7 +18222,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>1746.397</v>
@@ -18271,7 +18281,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>1747.352</v>
@@ -18330,7 +18340,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>1613.623</v>
@@ -18389,7 +18399,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>1768.589</v>
@@ -18448,7 +18458,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>1815.131</v>
@@ -18507,7 +18517,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>1611.452</v>
@@ -18566,7 +18576,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>1748.778</v>
@@ -18625,7 +18635,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>1707.036</v>
@@ -18684,7 +18694,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>1791.586</v>
@@ -18743,7 +18753,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>1636.534</v>
@@ -18802,7 +18812,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>1576.6</v>
@@ -18861,7 +18871,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>1726.218</v>
@@ -18920,7 +18930,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>1603.06</v>
@@ -18979,7 +18989,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>1648.291</v>
@@ -19038,7 +19048,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>1585.004</v>
@@ -19097,7 +19107,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>1695.759</v>
@@ -19156,7 +19166,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>1678.688</v>
@@ -19215,7 +19225,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>1646.907</v>
@@ -19274,7 +19284,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>1711.742</v>
@@ -19333,7 +19343,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>1749.92</v>
@@ -19392,7 +19402,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>1764.101</v>
@@ -19451,7 +19461,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>1716.211</v>
@@ -19510,7 +19520,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>1716.771</v>
@@ -19569,7 +19579,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>1002.737</v>
@@ -19628,7 +19638,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>450.131</v>
@@ -19687,7 +19697,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>879.061</v>
@@ -19746,7 +19756,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>1135.248</v>
@@ -19805,7 +19815,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>1242.176</v>
@@ -19864,7 +19874,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>1157.742</v>
@@ -19923,7 +19933,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>1173.011</v>
@@ -19982,7 +19992,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>1322.079</v>
@@ -20041,7 +20051,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>1502.255</v>
@@ -20100,7 +20110,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>1623.949</v>
@@ -20159,7 +20169,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>1623.219</v>
@@ -20218,7 +20228,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>1604.465</v>
@@ -20277,7 +20287,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>1737.766</v>
@@ -20336,7 +20346,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>1681.574</v>
@@ -20395,7 +20405,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>1416.126</v>
@@ -20454,7 +20464,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>1446.219</v>
@@ -20513,7 +20523,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>1787.34</v>
@@ -20572,7 +20582,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>1863.355</v>
@@ -20631,7 +20641,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>1843.839</v>
@@ -20690,7 +20700,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>1627.277</v>
@@ -20749,7 +20759,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>2038.872</v>
@@ -20808,7 +20818,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>2164.567</v>
@@ -20867,7 +20877,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>1881.662</v>
@@ -20926,7 +20936,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>1912.973</v>
@@ -20985,7 +20995,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>2053.229</v>
@@ -21044,7 +21054,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>2025.019</v>
@@ -21103,7 +21113,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>2082.902</v>
@@ -21162,7 +21172,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>1896.353</v>
@@ -21221,7 +21231,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>2269.559</v>
@@ -21280,7 +21290,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>2310.59</v>
@@ -21339,7 +21349,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>2203.499</v>
@@ -21398,7 +21408,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>2229.103</v>
@@ -21457,7 +21467,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>2145.135</v>
@@ -21516,7 +21526,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>2199.754</v>
@@ -21575,7 +21585,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>2154.778</v>
@@ -21634,7 +21644,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>1966.672</v>
@@ -21693,7 +21703,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>2093.089</v>
@@ -21752,7 +21762,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>2030.048</v>
@@ -21811,7 +21821,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>2093.185</v>
@@ -21870,7 +21880,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>2052.453</v>
@@ -21929,7 +21939,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>2228.824</v>
@@ -21988,7 +21998,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>2208.83</v>
@@ -22047,7 +22057,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>2060.076</v>
@@ -22106,7 +22116,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>2134.85</v>
@@ -22165,7 +22175,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>2077.061</v>
@@ -22224,7 +22234,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>2090.888</v>
@@ -22283,7 +22293,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>2082.022</v>
@@ -22342,7 +22352,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>1880.601</v>
@@ -22401,7 +22411,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>1929.30111543109</v>
@@ -22460,7 +22470,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>2012.81152656905</v>
@@ -22519,7 +22529,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>2166.37106446468</v>
@@ -22578,7 +22588,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>2094.75372592009</v>
@@ -22637,7 +22647,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>2233.01301983058</v>
@@ -22696,7 +22706,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>2060.79708181739</v>
@@ -22755,7 +22765,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>2125.52294225439</v>
@@ -22814,7 +22824,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>2188.10188755066</v>
@@ -22873,7 +22883,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>2208.46566419479</v>
@@ -22932,7 +22942,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>2189.08483072309</v>
@@ -22991,7 +23001,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>2055.395</v>
@@ -23050,7 +23060,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>1844.741</v>
@@ -23109,7 +23119,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>1934.043</v>
@@ -23168,7 +23178,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>1942.549</v>
@@ -23227,7 +23237,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>1973.266</v>
@@ -23286,7 +23296,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>1889.072</v>
@@ -23345,7 +23355,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>2006.227</v>
@@ -23404,7 +23414,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>1988.238</v>
@@ -23463,7 +23473,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>1983.375</v>
@@ -23522,7 +23532,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>2037.133</v>
@@ -23581,7 +23591,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>1949.769</v>
@@ -23640,7 +23650,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>2181.39</v>
@@ -23699,7 +23709,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>2267.271</v>
@@ -23758,7 +23768,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>2051.143</v>
@@ -23817,7 +23827,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>2303.894</v>
@@ -23876,7 +23886,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>2229.49</v>
@@ -23935,7 +23945,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2"/>
       <c r="C366" s="3" t="n">
@@ -23968,7 +23978,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3" t="n">
@@ -24001,7 +24011,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3" t="n">
@@ -24034,7 +24044,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3" t="n">
@@ -24067,7 +24077,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3" t="n">
@@ -24100,7 +24110,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3" t="n">
@@ -24133,7 +24143,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3" t="n">
@@ -24166,7 +24176,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3" t="n">
@@ -24199,7 +24209,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2"/>
       <c r="C374" s="3" t="n">
@@ -24232,7 +24242,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2"/>
       <c r="C375" s="3" t="n">
@@ -24265,7 +24275,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2"/>
       <c r="C376" s="3" t="n">
@@ -24298,7 +24308,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2"/>
       <c r="C377" s="3" t="n">
@@ -24331,7 +24341,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2"/>
       <c r="C378" s="3"/>
@@ -24354,7 +24364,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2"/>
       <c r="C379" s="3"/>
@@ -24377,7 +24387,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2"/>
       <c r="C380" s="3"/>
@@ -24400,7 +24410,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2"/>
       <c r="C381" s="3"/>
@@ -24423,7 +24433,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2"/>
       <c r="C382" s="3"/>
@@ -24446,7 +24456,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2"/>
       <c r="C383" s="3"/>
@@ -24469,7 +24479,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2"/>
       <c r="C384" s="3"/>
@@ -24492,7 +24502,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="3"/>
@@ -24515,7 +24525,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2"/>
       <c r="C386" s="3"/>
@@ -24538,7 +24548,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2"/>
       <c r="C387" s="3"/>
@@ -24561,7 +24571,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2"/>
       <c r="C388" s="3"/>
@@ -24584,7 +24594,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2"/>
       <c r="C389" s="3"/>
@@ -24607,7 +24617,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3"/>
@@ -24630,7 +24640,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3"/>
@@ -24653,7 +24663,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3"/>
@@ -24676,7 +24686,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3"/>
@@ -24699,7 +24709,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3"/>
@@ -24722,7 +24732,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3"/>
@@ -24745,7 +24755,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3"/>
@@ -24768,7 +24778,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3"/>
@@ -24791,7 +24801,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3"/>
@@ -24814,7 +24824,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3"/>
@@ -24837,7 +24847,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3"/>
@@ -24860,7 +24870,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3"/>
@@ -24883,7 +24893,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -24906,7 +24916,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -24929,7 +24939,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -24952,7 +24962,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -24975,7 +24985,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -24998,7 +25008,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25021,7 +25031,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25044,7 +25054,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25067,7 +25077,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25090,7 +25100,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -25113,7 +25123,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -25136,7 +25146,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -25159,7 +25169,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -25182,7 +25192,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -25205,7 +25215,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -25228,7 +25238,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -25251,7 +25261,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -25274,7 +25284,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -25297,7 +25307,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -25320,7 +25330,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -25354,97 +25364,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -25468,7 +25478,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -25478,160 +25488,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0160067374094991</v>
+        <v>-0.0158220910372178</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0117060620910076</v>
+        <v>0.0127899013555943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0151644414212752</v>
+        <v>0.016536348697969</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0284570563367201</v>
+        <v>0.0294622550358385</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.091028431434083</v>
+        <v>0.0926047761540446</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.170618164231167</v>
+        <v>0.171493022968696</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.238998163036501</v>
+        <v>0.237187979177776</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.288563117147436</v>
+        <v>0.285436233265778</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.335733407393288</v>
+        <v>0.333475021079591</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.343167902977312</v>
+        <v>0.341882879900403</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.306427893323006</v>
+        <v>0.305746042005264</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.272895558559665</v>
+        <v>0.272837794009525</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.242747552469495</v>
+        <v>0.243770015378361</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.211824992035485</v>
+        <v>0.213545287635328</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.188747648848119</v>
+        <v>0.190445399892825</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.121178422046143</v>
+        <v>0.122530989438816</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0297136676761131</v>
+        <v>0.0302910750884286</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.00310446317373542</v>
+        <v>-0.00275674750746945</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.00476294134073516</v>
+        <v>-0.00497436422477059</v>
       </c>
     </row>
     <row r="24">

</xml_diff>